<commit_message>
Fases 1-5 completas: extracción, clasificación, organización y watcher en tiempo real
</commit_message>
<xml_diff>
--- a/salida_prueba/FACTURAS/PENDIENTES/Registro_Pendientes.xlsx
+++ b/salida_prueba/FACTURAS/PENDIENTES/Registro_Pendientes.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:C2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -436,34 +436,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-07-12 15:37:55</t>
+          <t>2026-07-12 18:50:40</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>consorcio el milagro.jpeg</t>
+          <t>consorcio v y j.jpeg</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>RUC/nombre de consorcio no encontrado</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>2026-07-12 15:37:55</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>consorcio salud primavera.jpeg</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>RUC/nombre de consorcio no encontrado</t>
+          <t>Fecha de emisión no encontrada</t>
         </is>
       </c>
     </row>

</xml_diff>